<commit_message>
Optimize Mobile Schedule Viewer (Zooming & Dimensions)
</commit_message>
<xml_diff>
--- a/static/assets/section_template.xlsx
+++ b/static/assets/section_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WFH\jeremy\CvSU_Scheduling_System\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB6B4B38-679C-46DD-9730-4FC8C0FDAC53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C0D6737-6D35-4095-BB9F-712DE5D380C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1005" yWindow="1005" windowWidth="13620" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1200" windowWidth="12990" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Infotech" sheetId="1" r:id="rId1"/>
@@ -504,18 +504,15 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -523,17 +520,11 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -548,6 +539,15 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -594,6 +594,158 @@
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1123950" cy="1123950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="image1.jpg">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BA2C685A-BAA5-4F1F-A733-C31D5A42C09E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1123950" cy="1123950"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>638175</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1123950" cy="1123950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="image1.jpg">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E4EB2D23-6959-466B-88DE-F39FFE7A7A29}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4276725" y="1123950"/>
+          <a:ext cx="1123950" cy="1123950"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1009650</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1123950" cy="1123950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="image1.jpg">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{71640D13-CDEF-4C08-B68C-61A371AF0168}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3543300" y="2619375"/>
+          <a:ext cx="1123950" cy="1123950"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1123950" cy="1123950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="image1.jpg">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C42EB2B-A480-426B-B152-413BF3EF3867}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4953000" y="2124075"/>
+          <a:ext cx="1123950" cy="1123950"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
@@ -845,7 +997,7 @@
     </row>
     <row r="2" spans="1:26" ht="12" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="41" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="28"/>
@@ -875,7 +1027,7 @@
     </row>
     <row r="3" spans="1:26" ht="15" customHeight="1">
       <c r="A3" s="1"/>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="42" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="28"/>
@@ -905,7 +1057,7 @@
     </row>
     <row r="4" spans="1:26" ht="12" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="41" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="28"/>
@@ -935,7 +1087,7 @@
     </row>
     <row r="5" spans="1:26" ht="12" customHeight="1">
       <c r="A5" s="1"/>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="41" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="28"/>
@@ -965,7 +1117,7 @@
     </row>
     <row r="6" spans="1:26" ht="12" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="43" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="28"/>
@@ -995,7 +1147,7 @@
     </row>
     <row r="7" spans="1:26" ht="12" customHeight="1">
       <c r="A7" s="1"/>
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="33" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="28"/>
@@ -1025,7 +1177,7 @@
     </row>
     <row r="8" spans="1:26" ht="12" customHeight="1">
       <c r="A8" s="1"/>
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="33" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="28"/>
@@ -1083,15 +1235,15 @@
     </row>
     <row r="10" spans="1:26" ht="18" customHeight="1">
       <c r="A10" s="1"/>
-      <c r="B10" s="38"/>
-      <c r="C10" s="39"/>
+      <c r="B10" s="35"/>
+      <c r="C10" s="36"/>
       <c r="D10" s="5"/>
       <c r="E10" s="3"/>
       <c r="F10" s="6"/>
-      <c r="G10" s="40" t="s">
+      <c r="G10" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="H10" s="39"/>
+      <c r="H10" s="36"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
@@ -1113,14 +1265,14 @@
     </row>
     <row r="11" spans="1:26" ht="18" customHeight="1">
       <c r="A11" s="1"/>
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="42"/>
+      <c r="C11" s="39"/>
       <c r="D11" s="5"/>
       <c r="E11" s="3"/>
       <c r="F11" s="6"/>
-      <c r="G11" s="43" t="s">
+      <c r="G11" s="40" t="s">
         <v>9</v>
       </c>
       <c r="H11" s="28"/>
@@ -2173,16 +2325,16 @@
     </row>
     <row r="46" spans="1:26" ht="17.25" customHeight="1">
       <c r="A46" s="1"/>
-      <c r="B46" s="35" t="s">
+      <c r="B46" s="27" t="s">
         <v>46</v>
       </c>
       <c r="C46" s="28"/>
       <c r="D46" s="20"/>
-      <c r="E46" s="36" t="s">
+      <c r="E46" s="29" t="s">
         <v>47</v>
       </c>
       <c r="F46" s="28"/>
-      <c r="G46" s="37" t="s">
+      <c r="G46" s="30" t="s">
         <v>48</v>
       </c>
       <c r="H46" s="28"/>
@@ -2210,11 +2362,11 @@
       <c r="B47" s="28"/>
       <c r="C47" s="28"/>
       <c r="D47" s="22"/>
-      <c r="E47" s="32" t="s">
+      <c r="E47" s="31" t="s">
         <v>49</v>
       </c>
       <c r="F47" s="28"/>
-      <c r="G47" s="33" t="s">
+      <c r="G47" s="32" t="s">
         <v>50</v>
       </c>
       <c r="H47" s="28"/>
@@ -2356,7 +2508,10 @@
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
-      <c r="G52" s="34"/>
+      <c r="G52" s="34">
+        <f>B10</f>
+        <v>0</v>
+      </c>
       <c r="H52" s="28"/>
       <c r="I52" s="1"/>
       <c r="J52" s="1"/>
@@ -2491,12 +2646,12 @@
     </row>
     <row r="57" spans="1:26" ht="12.75" customHeight="1">
       <c r="A57" s="1"/>
-      <c r="B57" s="35"/>
+      <c r="B57" s="27"/>
       <c r="C57" s="28"/>
       <c r="D57" s="20"/>
-      <c r="E57" s="36"/>
+      <c r="E57" s="29"/>
       <c r="F57" s="28"/>
-      <c r="G57" s="37"/>
+      <c r="G57" s="30"/>
       <c r="H57" s="28"/>
       <c r="I57" s="1"/>
       <c r="J57" s="1"/>
@@ -2522,9 +2677,9 @@
       <c r="B58" s="28"/>
       <c r="C58" s="28"/>
       <c r="D58" s="22"/>
-      <c r="E58" s="32"/>
+      <c r="E58" s="31"/>
       <c r="F58" s="28"/>
-      <c r="G58" s="33"/>
+      <c r="G58" s="32"/>
       <c r="H58" s="28"/>
       <c r="I58" s="1"/>
       <c r="J58" s="1"/>
@@ -28923,11 +29078,11 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="B57:C58"/>
-    <mergeCell ref="E57:F57"/>
-    <mergeCell ref="G57:H57"/>
-    <mergeCell ref="E58:F58"/>
-    <mergeCell ref="G58:H58"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B6:H6"/>
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="B8:H8"/>
     <mergeCell ref="E47:F47"/>
@@ -28940,11 +29095,11 @@
     <mergeCell ref="B46:C47"/>
     <mergeCell ref="E46:F46"/>
     <mergeCell ref="G46:H46"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B57:C58"/>
+    <mergeCell ref="E57:F57"/>
+    <mergeCell ref="G57:H57"/>
+    <mergeCell ref="E58:F58"/>
+    <mergeCell ref="G58:H58"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B7" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>

</xml_diff>